<commit_message>
Access list updated via Admin Panel — 6/11/2026, 8:15:57 AM
</commit_message>
<xml_diff>
--- a/catch_dashboard_access.xlsx
+++ b/catch_dashboard_access.xlsx
@@ -1,121 +1,58 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jacec\Documents\CMC DATA SOLUTIONS\REFERENCE TABLES\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21940" windowHeight="8590"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Dashboard Access" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
-  <si>
-    <t>RowCount</t>
-  </si>
-  <si>
-    <t>FirstName</t>
-  </si>
-  <si>
-    <t>LastName</t>
-  </si>
-  <si>
-    <t>EmailAddress</t>
-  </si>
-  <si>
-    <t>Program</t>
-  </si>
-  <si>
-    <t>Janice</t>
-  </si>
-  <si>
-    <t>Sparks</t>
-  </si>
-  <si>
-    <t>janice.sparks@catchgh.org</t>
-  </si>
-  <si>
-    <t>ALL</t>
-  </si>
-  <si>
-    <t>Brandi</t>
-  </si>
-  <si>
-    <t>Smith</t>
-  </si>
-  <si>
-    <t>brandi.smith@houstontx.gov</t>
-  </si>
-  <si>
-    <t>Michael</t>
-  </si>
-  <si>
-    <t>Creary</t>
-  </si>
-  <si>
-    <t>creary.michael@digitaldataexperts.net</t>
-  </si>
-  <si>
-    <t>GUIDE</t>
-  </si>
-</sst>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <numFmts count="1">
+    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
+  </numFmts>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF1F4E79"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD6E4F0"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -123,56 +60,18 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFBFBFBF"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFBFBFBF"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFBFBFBF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFBFBFBF"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
 </styleSheet>
 </file>
 
@@ -251,6 +150,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -285,6 +185,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -319,20 +220,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -454,91 +351,125 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="32" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1">
+      <c r="A1" t="str">
+        <v>RowCount</v>
+      </c>
+      <c r="B1" t="str">
+        <v>FirstName</v>
+      </c>
+      <c r="C1" t="str">
+        <v>LastName</v>
+      </c>
+      <c r="D1" t="str">
+        <v>EmailAddress</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Program</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" t="str">
+        <v>Janice</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Sparks</v>
+      </c>
+      <c r="D2" t="str">
+        <v>janice.sparks@catchgh.org</v>
+      </c>
+      <c r="E2" t="str">
+        <v>ALL</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B3" t="str">
+        <v>Brandi</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Smith</v>
+      </c>
+      <c r="D3" t="str">
+        <v>brandi.smith@houstontx.gov</v>
+      </c>
+      <c r="E3" t="str">
+        <v>ALL</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="4">
-        <v>2</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="4">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>15</v>
+      <c r="B4" t="str">
+        <v>Michael</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Creary</v>
+      </c>
+      <c r="D4" t="str">
+        <v>creary.michael@digitaldataexperts.net</v>
+      </c>
+      <c r="E4" t="str">
+        <v>CHI</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>